<commit_message>
Changes related to the hero seciton
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -501,7 +501,7 @@
         <v>site.seatsPerVan</v>
       </c>
       <c r="B12">
-        <v>12</v>
+        <v>25</v>
       </c>
     </row>
     <row r="13">
@@ -509,7 +509,7 @@
         <v>nextDeparture.month</v>
       </c>
       <c r="B13" t="str">
-        <v>August</v>
+        <v>September</v>
       </c>
     </row>
     <row r="14">
@@ -517,7 +517,7 @@
         <v>nextDeparture.seatsLeft</v>
       </c>
       <c r="B14">
-        <v>3</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -529,7 +529,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F22"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -791,16 +791,196 @@
         <v>https://www.flickr.com/photos/22539273@N00/55898931</v>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>tours/islamabad.jpg</v>
+      </c>
+      <c r="B14" t="str">
+        <v>The Shah Faisal Mosque, Islamabad</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Mansoor Bashir</v>
+      </c>
+      <c r="D14" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E14" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0/</v>
+      </c>
+      <c r="F14" t="str">
+        <v>https://commons.wikimedia.org/w/index.php?curid=62674975</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>tours/muzaffarabad.jpg</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Muzaffarabad city, Azad Kashmir 2019-06-07</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Mariaivon</v>
+      </c>
+      <c r="D15" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E15" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0/</v>
+      </c>
+      <c r="F15" t="str">
+        <v>https://commons.wikimedia.org/w/index.php?curid=87078678</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>tours/keran.jpg</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Keran Village of Neelum Valley AJK Northern Pakistan</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Syed Ali Zaidi 1167</v>
+      </c>
+      <c r="D16" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E16" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0/</v>
+      </c>
+      <c r="F16" t="str">
+        <v>https://commons.wikimedia.org/w/index.php?curid=69094679</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>tours/kel.jpg</v>
+      </c>
+      <c r="B17" t="str">
+        <v>A Stream of River Neelum at Kel, Neelum Valley Road, Pakistan controlled Kashmir</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Ijazurrehman1970</v>
+      </c>
+      <c r="D17" t="str">
+        <v>CC BY-SA 3.0</v>
+      </c>
+      <c r="E17" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/3.0/</v>
+      </c>
+      <c r="F17" t="str">
+        <v>https://commons.wikimedia.org/w/index.php?curid=40356744</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>tours/arang-kel.jpg</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Arang Kel, Neelum Valley, Azad Jammu &amp; Kashmir, Pakistan</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Nadeem Riaz</v>
+      </c>
+      <c r="D18" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E18" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0/</v>
+      </c>
+      <c r="F18" t="str">
+        <v>https://commons.wikimedia.org/w/index.php?curid=59237123</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>hero/winter.jpg</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Nanga Parbat The Killer Mountain</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Tahsin Anwar Ali</v>
+      </c>
+      <c r="D19" t="str">
+        <v>CC BY-SA 3.0</v>
+      </c>
+      <c r="E19" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/3.0/</v>
+      </c>
+      <c r="F19" t="str">
+        <v>https://commons.wikimedia.org/w/index.php?curid=40616492</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>hero/spring.jpg</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Keran Village of Neelum Valley AJK Northern Pakistan</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Syed Ali Zaidi 1167</v>
+      </c>
+      <c r="D20" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E20" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0/</v>
+      </c>
+      <c r="F20" t="str">
+        <v>https://commons.wikimedia.org/w/index.php?curid=69094679</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>hero/summer.jpg</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Arang Kel, Neelum Valley, Azad Jammu &amp; Kashmir, Pakistan</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Nadeem Riaz</v>
+      </c>
+      <c r="D21" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E21" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0/</v>
+      </c>
+      <c r="F21" t="str">
+        <v>https://commons.wikimedia.org/w/index.php?curid=59237123</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>hero/autumn.jpg</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Autumn in Hunza Valley</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Ghezwan274</v>
+      </c>
+      <c r="D22" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E22" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0/</v>
+      </c>
+      <c r="F22" t="str">
+        <v>https://commons.wikimedia.org/w/index.php?curid=69010681</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F22"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S3"/>
+  <dimension ref="A1:S2"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -863,22 +1043,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>kalam-mahodand-lake</v>
+        <v>arang-kel-neelum-valley</v>
       </c>
       <c r="B2" t="str">
-        <v>Kalam &amp; Mahodand Lake</v>
+        <v>Arang Kel &amp; the Neelum Valley</v>
       </c>
       <c r="C2" t="str">
-        <v>8–9 August</v>
+        <v>28–29 September</v>
       </c>
       <c r="D2" t="str">
-        <v>8 Aug</v>
+        <v>28 Sep</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-08-08</v>
+        <v>2026-09-28</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-08-09</v>
+        <v>2026-09-29</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -890,105 +1070,46 @@
         <v>7999</v>
       </c>
       <c r="J2">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="K2">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="L2" t="str">
-        <v>kalam.jpg</v>
+        <v>arang-kel.jpg</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>One night at 2,743 m</v>
       </c>
       <c r="N2" t="str">
-        <v>Swat Valley, Khyber Pakhtunkhwa</v>
+        <v>Neelum Valley, Azad Kashmir</v>
       </c>
       <c r="O2">
-        <v>2865</v>
+        <v>2743</v>
       </c>
       <c r="P2" t="str">
-        <v>Two days up the Swat valley, ending on the jeep track to a lake that sits just under 2,900 metres.</v>
+        <v>Two days up the Neelum valley, ending with a chairlift over the river and a climb to a meadow with no road into it.</v>
       </c>
       <c r="Q2" t="str">
-        <v>Van from Islamabad and back | One night in Kalam | Breakfast both days | Jeep up the Mahodand track</v>
+        <v>Van from Islamabad and back | One night in Arang Kel | Breakfast both days | Chairlift across the Neelum</v>
       </c>
       <c r="R2" t="str">
-        <v>Swat Valley | Bahrain Bazaar | Blue Point | Mahodand Lake</v>
+        <v>Muzaffarabad | Keran | Kel | Arang Kel</v>
       </c>
       <c r="S2" t="str">
-        <v>Lunch and dinner | Boat hire at the lake | Anything you buy at the bazaar</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Fairy Meadows &amp; Nanga Parbat Base Camp</v>
-      </c>
-      <c r="C3" t="str">
-        <v>23–27 August</v>
-      </c>
-      <c r="D3" t="str">
-        <v>23 Aug</v>
-      </c>
-      <c r="E3" t="str">
-        <v>2026-08-23</v>
-      </c>
-      <c r="F3" t="str">
-        <v>2026-08-27</v>
-      </c>
-      <c r="G3">
-        <v>4</v>
-      </c>
-      <c r="H3">
-        <v>5</v>
-      </c>
-      <c r="I3">
-        <v>14999</v>
-      </c>
-      <c r="J3">
-        <v>12</v>
-      </c>
-      <c r="K3">
-        <v>5</v>
-      </c>
-      <c r="L3" t="str">
-        <v>fairy-meadows.jpg</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Holi colours at the meadows</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Diamer, Gilgit-Baltistan</v>
-      </c>
-      <c r="O3">
-        <v>4600</v>
-      </c>
-      <c r="P3" t="str">
-        <v>Five days to walk up to the foot of the ninth highest mountain on earth, sleeping at 3,300 metres.</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>Pickup and drop, Islamabad | Four nights at the meadows | All meals | Jeep up the Raikot track</v>
-      </c>
-      <c r="R3" t="str">
-        <v>Fairy Meadows | Nanga Parbat Base Camp</v>
-      </c>
-      <c r="S3" t="str">
-        <v>Porters for personal bags | Anything bought on the highway | Gear hire</v>
+        <v>Lunch and dinner | Horses up the ridge | Anything you buy in the bazaar</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S2"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:G6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1004,15 +1125,18 @@
         <v>day</v>
       </c>
       <c r="E1" t="str">
+        <v>img</v>
+      </c>
+      <c r="F1" t="str">
         <v>note</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>does</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>kalam-mahodand-lake</v>
+        <v>arang-kel-neelum-valley</v>
       </c>
       <c r="B2" t="str">
         <v>Islamabad</v>
@@ -1024,222 +1148,117 @@
         <v>Day 1 · 00:00</v>
       </c>
       <c r="E2" t="str">
+        <v>islamabad.jpg</v>
+      </c>
+      <c r="F2" t="str">
         <v>Midnight pickup — the driving happens while you sleep.</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>Pickup points shared in the trip group | Seats allotted, bags loaded, lights off</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>kalam-mahodand-lake</v>
+        <v>arang-kel-neelum-valley</v>
       </c>
       <c r="B3" t="str">
-        <v>Mingora</v>
+        <v>Muzaffarabad</v>
       </c>
       <c r="C3">
-        <v>980</v>
+        <v>737</v>
       </c>
       <c r="D3" t="str">
-        <v>Day 1 · morning</v>
+        <v>Day 1 · 04:30</v>
       </c>
       <c r="E3" t="str">
-        <v>Breakfast past Mardan, then into the Swat valley.</v>
+        <v>muzaffarabad.jpg</v>
       </c>
       <c r="F3" t="str">
-        <v>Breakfast stop on the way up | The climb up the Swat valley begins</v>
+        <v>Breakfast where the Neelum meets the Jhelum, as the light comes up.</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Breakfast stop | ID cards out — there are checkposts up the valley</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>kalam-mahodand-lake</v>
+        <v>arang-kel-neelum-valley</v>
       </c>
       <c r="B4" t="str">
-        <v>Bahrain</v>
+        <v>Keran</v>
       </c>
       <c r="C4">
-        <v>1400</v>
+        <v>1372</v>
       </c>
       <c r="D4" t="str">
-        <v>Day 1 · midday</v>
+        <v>Day 1 · 09:00</v>
       </c>
       <c r="E4" t="str">
-        <v>An hour at Bahrain bazaar, on the river.</v>
+        <v>keran.jpg</v>
       </c>
       <c r="F4" t="str">
-        <v>Walk the bazaar | Tea by the Swat river</v>
+        <v>Tea on the bank of the Neelum, the far side of the river in Indian-administered Kashmir.</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Tea and a walk along the water | The valley road narrows from here</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>kalam-mahodand-lake</v>
+        <v>arang-kel-neelum-valley</v>
       </c>
       <c r="B5" t="str">
-        <v>Kalam</v>
+        <v>Kel</v>
       </c>
       <c r="C5">
-        <v>2000</v>
+        <v>2097</v>
       </c>
       <c r="D5" t="str">
-        <v>Day 1 · evening</v>
+        <v>Day 1 · 14:00</v>
       </c>
       <c r="E5" t="str">
-        <v>Blue Point in the afternoon, beds in Kalam by dark.</v>
+        <v>kel.jpg</v>
       </c>
       <c r="F5" t="str">
-        <v>Blue Point viewpoint | One night in Kalam — included | Breakfast in the morning</v>
+        <v>The van's last stop. From here it is the chairlift and your own legs.</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Van parks at Kel | Chairlift across the Neelum — included | The climb up to the meadow</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>kalam-mahodand-lake</v>
+        <v>arang-kel-neelum-valley</v>
       </c>
       <c r="B6" t="str">
-        <v>Mahodand</v>
+        <v>Arang Kel</v>
       </c>
       <c r="C6">
-        <v>2865</v>
+        <v>2743</v>
       </c>
       <c r="D6" t="str">
-        <v>Day 2</v>
+        <v>Days 1–2 · 16:00</v>
       </c>
       <c r="E6" t="str">
-        <v>Out early up the jeep track to the lake — rough, and that is the point.</v>
+        <v>arang-kel.jpg</v>
       </c>
       <c r="F6" t="str">
-        <v>Jeep up the Mahodand track — included | Time at the lake (boat hire extra) | Lunch, then the drive home the same night</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Islamabad</v>
-      </c>
-      <c r="C7">
-        <v>540</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Day 1 · before dawn</v>
-      </c>
-      <c r="E7" t="str">
-        <v>Out of Islamabad in the dark and onto the Karakoram Highway.</v>
-      </c>
-      <c r="F7" t="str">
-        <v>Pickup points shared in the trip group | Onto the KKH before the traffic</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Chilas</v>
-      </c>
-      <c r="C8">
-        <v>1265</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Day 1 · evening</v>
-      </c>
-      <c r="E8" t="str">
-        <v>A full day of driving along the Indus ends here.</v>
-      </c>
-      <c r="F8" t="str">
-        <v>Stops along the Indus gorge | End of the first day on the road</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Raikot Bridge</v>
-      </c>
-      <c r="C9">
-        <v>1180</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Day 2 · morning</v>
-      </c>
-      <c r="E9" t="str">
-        <v>The van stays here. Jeeps take over for the Raikot track.</v>
-      </c>
-      <c r="F9" t="str">
-        <v>Switch to jeeps — included | One of the more committing roads in the country</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Tato</v>
-      </c>
-      <c r="C10">
-        <v>2600</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Day 2</v>
-      </c>
-      <c r="E10" t="str">
-        <v>The jeep road ends. The walk in to the meadows starts.</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Jeeps drop you at the trailhead | Walk in to Fairy Meadows</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Fairy Meadows</v>
-      </c>
-      <c r="C11">
-        <v>3300</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Days 2–4</v>
-      </c>
-      <c r="E11" t="str">
-        <v>Home for four nights, facing Nanga Parbat.</v>
-      </c>
-      <c r="F11" t="str">
-        <v>Camp goes up, Holi colours in the evening | Beyal camp on the morning of day 4 | All meals included</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Base Camp</v>
-      </c>
-      <c r="C12">
-        <v>4600</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Day 3</v>
-      </c>
-      <c r="E12" t="str">
-        <v>The long day — up to Nanga Parbat Base Camp and back before dark.</v>
-      </c>
-      <c r="F12" t="str">
-        <v>Walk slowly, drink more water than you think | Back at the meadows by nightfall</v>
+        <v>A green shelf above the valley — wooden huts, pine forest, and no road in.</v>
+      </c>
+      <c r="G6" t="str">
+        <v>One night in a hut — included | Breakfast in the morning | The meadow before the day trippers arrive</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F12"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1254,84 +1273,29 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>kalam-mahodand-lake</v>
+        <v>arang-kel-neelum-valley</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>Midnight departure from Islamabad. Breakfast somewhere past Mardan, then the climb up the Swat valley. An hour at Bahrain bazaar, Blue Point in the afternoon, beds in Kalam by dark.</v>
+        <v>Midnight departure from Islamabad. Breakfast at Muzaffarabad as the light comes up, then the Neelum valley road all day — tea at Keran, lunch past Sharda. Kel by mid-afternoon, the chairlift across the river, and the last stretch up on foot. Night in a hut at Arang Kel.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>kalam-mahodand-lake</v>
+        <v>arang-kel-neelum-valley</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="str">
-        <v>Out early for the jeep track — it is rough, and that is the point. Time at Mahodand lake, lunch, then the long drive back down. Islamabad the same night.</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Out of Islamabad in the dark and onto the Karakoram Highway. A full day of driving along the Indus to Chilas.</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5" t="str">
-        <v>The Raikot jeep track — one of the more committing roads in the country — then the walk in to Fairy Meadows. Camp goes up, and the Holi colours come out in the evening.</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B6">
-        <v>3</v>
-      </c>
-      <c r="C6" t="str">
-        <v>The long day: up to Nanga Parbat Base Camp at 4,600 m and back down to the meadows before dark. Go slow, drink water.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B7">
-        <v>4</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Beyal camp in the morning, the rest of the day free at the meadows, then down to the jeeps and south along the Indus.</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>fairy-meadows-nanga-parbat</v>
-      </c>
-      <c r="B8">
-        <v>5</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Back in Islamabad.</v>
+        <v>Out early for the meadow before the day trippers come up. Down the ridge by late morning, back into the van at Kel, and the long drive home. Islamabad the same night.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C3"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1361,7 +1325,7 @@
         <v>Pay the advance</v>
       </c>
       <c r="B3" t="str">
-        <v>A seat is yours once the advance is in — vans are small and August fills early.</v>
+        <v>A seat is yours once the advance is in — vans are small and September fills early.</v>
       </c>
     </row>
     <row r="4">
@@ -1515,7 +1479,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1533,91 +1497,133 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>mahodand.jpg</v>
+        <v>arang-kel.jpg</v>
       </c>
       <c r="B2" t="str">
-        <v>Mahodand Lake</v>
+        <v>Arang Kel</v>
       </c>
       <c r="C2" t="str">
-        <v>Kalam</v>
+        <v>Neelum Valley</v>
       </c>
       <c r="D2">
-        <v>2865</v>
+        <v>2743</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>kumrat-river.jpg</v>
+        <v>keran.jpg</v>
       </c>
       <c r="B3" t="str">
-        <v>River camp</v>
+        <v>Keran</v>
       </c>
       <c r="C3" t="str">
-        <v>Kumrat</v>
+        <v>Neelum Valley</v>
       </c>
       <c r="D3">
-        <v>2300</v>
+        <v>1372</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>nanga-parbat.jpg</v>
+        <v>kel.jpg</v>
       </c>
       <c r="B4" t="str">
-        <v>Nanga Parbat</v>
+        <v>Kel</v>
       </c>
       <c r="C4" t="str">
-        <v>Diamer</v>
+        <v>Neelum Valley</v>
       </c>
       <c r="D4">
-        <v>8126</v>
+        <v>2097</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>saiful-muluk.jpg</v>
+        <v>mahodand.jpg</v>
       </c>
       <c r="B5" t="str">
-        <v>Saif-ul-Malook</v>
+        <v>Mahodand Lake</v>
       </c>
       <c r="C5" t="str">
-        <v>Naran</v>
+        <v>Kalam</v>
       </c>
       <c r="D5">
-        <v>3224</v>
+        <v>2865</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>kalash-people.jpg</v>
+        <v>kumrat-river.jpg</v>
       </c>
       <c r="B6" t="str">
-        <v>Bumburet</v>
+        <v>River camp</v>
       </c>
       <c r="C6" t="str">
-        <v>Chitral</v>
+        <v>Kumrat</v>
       </c>
       <c r="D6">
-        <v>1900</v>
+        <v>2300</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
+        <v>nanga-parbat.jpg</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Nanga Parbat</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Diamer</v>
+      </c>
+      <c r="D7">
+        <v>8126</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>saiful-muluk.jpg</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Saif-ul-Malook</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Naran</v>
+      </c>
+      <c r="D8">
+        <v>3224</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>kalash-people.jpg</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Bumburet</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Chitral</v>
+      </c>
+      <c r="D9">
+        <v>1900</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
         <v>ganga-choti.jpg</v>
       </c>
-      <c r="B7" t="str">
+      <c r="B10" t="str">
         <v>Ganga Choti</v>
       </c>
-      <c r="C7" t="str">
+      <c r="C10" t="str">
         <v>Bagh</v>
       </c>
-      <c r="D7">
+      <c r="D10">
         <v>3044</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1663,7 +1669,7 @@
         <v>How do I hold a seat?</v>
       </c>
       <c r="B5" t="str">
-        <v>Message the number. A seat is yours once the advance is in — vans are small and August fills early.</v>
+        <v>Message the number. A seat is yours once the advance is in — vans are small and September fills early.</v>
       </c>
     </row>
     <row r="6">
@@ -1679,7 +1685,7 @@
         <v>How high do we actually go, and does that matter?</v>
       </c>
       <c r="B7" t="str">
-        <v>Kalam tops out at 2,865 m, which nobody feels. Nanga Parbat Base Camp is 4,600 m, high enough that you walk slowly, drink more water than you think you need, and tell me if your head hurts.</v>
+        <v>Arang Kel tops out at 2,743 m, which nobody feels. The climb up from Kel is the part your legs notice, not your lungs — an hour or so on foot once the chairlift has taken you over the river.</v>
       </c>
     </row>
     <row r="8">
@@ -1687,7 +1693,7 @@
         <v>What should I bring?</v>
       </c>
       <c r="B8" t="str">
-        <v>A warm layer even in August, shoes you can walk a jeep track in, a power bank, your ID card, and any medicine you take. A full list goes out in the group before we leave.</v>
+        <v>A warm layer — it drops close to freezing up there at night in late September — shoes you can walk a rough track in, a power bank, your ID card, and any medicine you take. A full list goes out in the group before we leave.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes related to the booking
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -469,7 +469,7 @@
         <v>site.phone</v>
       </c>
       <c r="B8" t="str">
-        <v>+92 336 3202576</v>
+        <v>+92 305 1786177</v>
       </c>
     </row>
     <row r="9">
@@ -477,7 +477,7 @@
         <v>site.wa</v>
       </c>
       <c r="B9" t="str">
-        <v>https://wa.me/923363202576</v>
+        <v>https://wa.me/+923051786177</v>
       </c>
     </row>
     <row r="10">
@@ -1325,7 +1325,7 @@
         <v>Pay the advance</v>
       </c>
       <c r="B3" t="str">
-        <v>A seat is yours once the advance is in — vans are small and September fills early.</v>
+        <v>A seat is yours once the advance is in — trips are small and September fills early.</v>
       </c>
     </row>
     <row r="4">
@@ -1669,7 +1669,7 @@
         <v>How do I hold a seat?</v>
       </c>
       <c r="B5" t="str">
-        <v>Message the number. A seat is yours once the advance is in — vans are small and September fills early.</v>
+        <v>Message the number. A seat is yours once the advance is in — trips are small and September fills early.</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
Changes related to the about us page
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -13,6 +13,7 @@
     <sheet name="faqs" sheetId="8" r:id="rId8"/>
     <sheet name="reviews" sheetId="9" r:id="rId9"/>
     <sheet name="credits" sheetId="10" r:id="rId10"/>
+    <sheet name="about" sheetId="11" r:id="rId11"/>
   </sheets>
 </workbook>
 </file>
@@ -978,6 +979,272 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:E15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>block</v>
+      </c>
+      <c r="B1" t="str">
+        <v>name</v>
+      </c>
+      <c r="C1" t="str">
+        <v>role</v>
+      </c>
+      <c r="D1" t="str">
+        <v>text</v>
+      </c>
+      <c r="E1" t="str">
+        <v>photo</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>heading</v>
+      </c>
+      <c r="B2" t="str">
+        <v/>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+      <c r="D2" t="str">
+        <v>Northern Pakistan, planned and managed for you</v>
+      </c>
+      <c r="E2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>description</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v/>
+      </c>
+      <c r="D3" t="str">
+        <v>Travel With Wahid plans and manages trips from Islamabad to northern Pakistan — fixed departures, custom group trips, and online booking with live seat availability.</v>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>story</v>
+      </c>
+      <c r="B4" t="str">
+        <v/>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+      <c r="D4" t="str">
+        <v>Travel With Wahid runs trips from Islamabad to the valleys of northern Pakistan — the Neelum valley and Arang Kel, Swat and Kalam, Fairy Meadows, Kumrat, Naran and the Kalash valleys.</v>
+      </c>
+      <c r="E4" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>story</v>
+      </c>
+      <c r="B5" t="str">
+        <v/>
+      </c>
+      <c r="C5" t="str">
+        <v/>
+      </c>
+      <c r="D5" t="str">
+        <v>We manage the whole trip: the route and timings, transport, stays and the day-by-day plan, with support on the road from pickup to drop-off. All you have to do is turn up.</v>
+      </c>
+      <c r="E5" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>story</v>
+      </c>
+      <c r="B6" t="str">
+        <v/>
+      </c>
+      <c r="C6" t="str">
+        <v/>
+      </c>
+      <c r="D6" t="str">
+        <v>Booking takes a few minutes online. See how many seats are left on a departure in real time, get a booking reference straight away, and check your booking status any time with your email.</v>
+      </c>
+      <c r="E6" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>story</v>
+      </c>
+      <c r="B7" t="str">
+        <v/>
+      </c>
+      <c r="C7" t="str">
+        <v/>
+      </c>
+      <c r="D7" t="str">
+        <v>Travelling as a university society, a batch, a family or a group of friends? We build custom trips around your dates, your group and your budget.</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>service</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Trip management</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
+      </c>
+      <c r="D8" t="str">
+        <v>Routes, transport, stays and timings planned and run for you, with support on the road from pickup to drop-off.</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>service</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Custom group trips</v>
+      </c>
+      <c r="C9" t="str">
+        <v/>
+      </c>
+      <c r="D9" t="str">
+        <v>Private trips for societies, batches, families and friends, built around your dates, group size and budget.</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>service</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Fixed departures</v>
+      </c>
+      <c r="C10" t="str">
+        <v/>
+      </c>
+      <c r="D10" t="str">
+        <v>Scheduled trips with a fixed date and a fixed price, and everything a seat covers written on the trip.</v>
+      </c>
+      <c r="E10" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>service</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Online booking</v>
+      </c>
+      <c r="C11" t="str">
+        <v/>
+      </c>
+      <c r="D11" t="str">
+        <v>Hold a seat on any departure online, send the advance receipt on WhatsApp, and get a booking reference straight away.</v>
+      </c>
+      <c r="E11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>service</v>
+      </c>
+      <c r="B12" t="str">
+        <v>Live seats and booking status</v>
+      </c>
+      <c r="C12" t="str">
+        <v/>
+      </c>
+      <c r="D12" t="str">
+        <v>See how many seats are left on every trip in real time, and look up your booking any time with your email.</v>
+      </c>
+      <c r="E12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>service</v>
+      </c>
+      <c r="B13" t="str">
+        <v>Trip group updates</v>
+      </c>
+      <c r="C13" t="str">
+        <v/>
+      </c>
+      <c r="D13" t="str">
+        <v>New dates and last-minute seats are posted first in the WhatsApp trip group.</v>
+      </c>
+      <c r="E13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>team</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Wahid</v>
+      </c>
+      <c r="C14" t="str">
+        <v>Founder &amp; trip lead</v>
+      </c>
+      <c r="D14" t="str">
+        <v>Founded Travel With Wahid and leads the trips — planning routes, managing departures and looking after every group on the road.</v>
+      </c>
+      <c r="E14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>team</v>
+      </c>
+      <c r="B15" t="str">
+        <v>Kamran Jesar</v>
+      </c>
+      <c r="C15" t="str">
+        <v>Tech Director</v>
+      </c>
+      <c r="D15" t="str">
+        <v>Built and runs the technology behind the trips — this website, the online booking system, live seat tracking and booking records.</v>
+      </c>
+      <c r="E15" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+  </ignoredErrors>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:S2"/>

</xml_diff>

<commit_message>
changes related to the contact and trip details
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -510,7 +510,7 @@
         <v>nextDeparture.month</v>
       </c>
       <c r="B13" t="str">
-        <v>September</v>
+        <v>October</v>
       </c>
     </row>
     <row r="14">
@@ -518,7 +518,7 @@
         <v>nextDeparture.seatsLeft</v>
       </c>
       <c r="B14">
-        <v>25</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -981,7 +981,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1209,16 +1209,16 @@
         <v>team</v>
       </c>
       <c r="B14" t="str">
-        <v>Wahid</v>
+        <v>Abdul Wahid</v>
       </c>
       <c r="C14" t="str">
-        <v>Founder &amp; trip lead</v>
+        <v>CEO &amp; Founder</v>
       </c>
       <c r="D14" t="str">
         <v>Founded Travel With Wahid and leads the trips — planning routes, managing departures and looking after every group on the road.</v>
       </c>
       <c r="E14" t="str">
-        <v/>
+        <v>/img/team/abdul-wahid.jpg</v>
       </c>
     </row>
     <row r="15">
@@ -1235,12 +1235,29 @@
         <v>Built and runs the technology behind the trips — this website, the online booking system, live seat tracking and booking records.</v>
       </c>
       <c r="E15" t="str">
-        <v/>
+        <v>/img/team/kamran-jesar.png</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>team</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Jan Muhammad Hur</v>
+      </c>
+      <c r="C16" t="str">
+        <v>Managing Director</v>
+      </c>
+      <c r="D16" t="str">
+        <v>A visionary leader with a passion for exploration and a commitment to creating memorable experiences.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>/img/team/jan-muhammad-hur.jpg</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E15"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1310,22 +1327,22 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>arang-kel-neelum-valley</v>
+        <v>naran-kaghan-babusar-top</v>
       </c>
       <c r="B2" t="str">
-        <v>Arang Kel &amp; the Neelum Valley</v>
+        <v>Naran, Kaghan &amp; Babusar Top</v>
       </c>
       <c r="C2" t="str">
-        <v>28–29 September</v>
+        <v>3–4 October</v>
       </c>
       <c r="D2" t="str">
-        <v>28 Sep</v>
+        <v>3 Oct</v>
       </c>
       <c r="E2" t="str">
-        <v>2026-09-28</v>
+        <v>2026-10-03</v>
       </c>
       <c r="F2" t="str">
-        <v>2026-09-29</v>
+        <v>2026-10-04</v>
       </c>
       <c r="G2">
         <v>1</v>
@@ -1340,31 +1357,31 @@
         <v>25</v>
       </c>
       <c r="K2">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="L2" t="str">
-        <v>arang-kel.jpg</v>
+        <v>naran.jpg</v>
       </c>
       <c r="M2" t="str">
-        <v>One night at 2,743 m</v>
+        <v>4 tickets booked</v>
       </c>
       <c r="N2" t="str">
-        <v>Neelum Valley, Azad Kashmir</v>
+        <v>Kaghan Valley, Khyber Pakhtunkhwa</v>
       </c>
       <c r="O2">
-        <v>2743</v>
+        <v>4173</v>
       </c>
       <c r="P2" t="str">
-        <v>Two days up the Neelum valley, ending with a chairlift over the river and a climb to a meadow with no road into it.</v>
+        <v>Two days up the Kaghan valley — Saif ul Malook, a night in Naran, Lulusar Lake and the snow at Babusar Top.</v>
       </c>
       <c r="Q2" t="str">
-        <v>Van from Islamabad and back | One night in Arang Kel | Breakfast both days | Chairlift across the Neelum</v>
+        <v>Transport from Islamabad and back | One night's accommodation in Naran | Breakfast on day 1 | Dinner at Balakot on day 2 | Toll taxes | Tour guide | Videography | First aid</v>
       </c>
       <c r="R2" t="str">
-        <v>Muzaffarabad | Keran | Kel | Arang Kel</v>
+        <v>Hazara Motorway | Balakot | Kiwai Waterfall | Paras | Kunhar River | Kaghan Valley | Naran | Naran Bazaar | Rafting Club | Saif ul Malook Lake | Batakundi | Lulusar Lake | Jalkhand | Besar | Babusar Top</v>
       </c>
       <c r="S2" t="str">
-        <v>Lunch and dinner | Horses up the ridge | Anything you buy in the bazaar</v>
+        <v>Jeep to Saif ul Malook Lake | Dinner in Naran on day 1 | Breakfast at Batakundi on day 2 | Rafting and zipline | Anything you buy in the bazaar</v>
       </c>
     </row>
   </sheetData>
@@ -1376,7 +1393,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:G9"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1403,7 +1420,7 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>arang-kel-neelum-valley</v>
+        <v>naran-kaghan-babusar-top</v>
       </c>
       <c r="B2" t="str">
         <v>Islamabad</v>
@@ -1412,113 +1429,182 @@
         <v>540</v>
       </c>
       <c r="D2" t="str">
-        <v>Day 1 · 00:00</v>
+        <v>Day 1 · 06:00</v>
       </c>
       <c r="E2" t="str">
         <v>islamabad.jpg</v>
       </c>
       <c r="F2" t="str">
-        <v>Midnight pickup — the driving happens while you sleep.</v>
+        <v>Report at 5:30 AM — the van leaves at 6:00 sharp from Quaid-e-Azam University.</v>
       </c>
       <c r="G2" t="str">
-        <v>Pickup points shared in the trip group | Seats allotted, bags loaded, lights off</v>
+        <v>Pickups: QAU, Kashmir Chowk, Abpara, G-8, H-9, G-13, 26 Number | Up the Hazara Motorway, breakfast stop at 9:30 — included</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>arang-kel-neelum-valley</v>
+        <v>naran-kaghan-babusar-top</v>
       </c>
       <c r="B3" t="str">
-        <v>Muzaffarabad</v>
+        <v>Naran</v>
       </c>
       <c r="C3">
-        <v>737</v>
+        <v>2409</v>
       </c>
       <c r="D3" t="str">
-        <v>Day 1 · 04:30</v>
+        <v>Day 1 · 13:00</v>
       </c>
       <c r="E3" t="str">
-        <v>muzaffarabad.jpg</v>
+        <v>naran.jpg</v>
       </c>
       <c r="F3" t="str">
-        <v>Breakfast where the Neelum meets the Jhelum, as the light comes up.</v>
+        <v>Into Naran by one, back again in the afternoon for the river and the bazaar.</v>
       </c>
       <c r="G3" t="str">
-        <v>Breakfast stop | ID cards out — there are checkposts up the valley</v>
+        <v>Rafting and zipline on the Kunhar at 4:00 PM | Hotel check-in at 6:00 PM — included | Naran Bazaar and dinner, 7–9 PM, at your own expense</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>arang-kel-neelum-valley</v>
+        <v>naran-kaghan-babusar-top</v>
       </c>
       <c r="B4" t="str">
-        <v>Keran</v>
+        <v>Saif ul Malook</v>
       </c>
       <c r="C4">
-        <v>1372</v>
+        <v>3224</v>
       </c>
       <c r="D4" t="str">
-        <v>Day 1 · 09:00</v>
+        <v>Day 1 · 13:30</v>
       </c>
       <c r="E4" t="str">
-        <v>keran.jpg</v>
+        <v>saiful-muluk.jpg</v>
       </c>
       <c r="F4" t="str">
-        <v>Tea on the bank of the Neelum, the far side of the river in Indian-administered Kashmir.</v>
+        <v>By jeep up to the lake, under Malika Parbat. Back in Naran by 3:30.</v>
       </c>
       <c r="G4" t="str">
-        <v>Tea and a walk along the water | The valley road narrows from here</v>
+        <v>Jeeps from Naran, 1:00–1:30 PM — not included | Time at the lake</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>arang-kel-neelum-valley</v>
+        <v>naran-kaghan-babusar-top</v>
       </c>
       <c r="B5" t="str">
-        <v>Kel</v>
+        <v>Batakundi</v>
       </c>
       <c r="C5">
-        <v>2097</v>
+        <v>2600</v>
       </c>
       <c r="D5" t="str">
-        <v>Day 1 · 14:00</v>
+        <v>Day 2 · 06:30</v>
       </c>
       <c r="E5" t="str">
-        <v>kel.jpg</v>
+        <v/>
       </c>
       <c r="F5" t="str">
-        <v>The van's last stop. From here it is the chairlift and your own legs.</v>
+        <v>Wake-up call at five, on the road by half past, breakfast up the valley.</v>
       </c>
       <c r="G5" t="str">
-        <v>Van parks at Kel | Chairlift across the Neelum — included | The climb up to the meadow</v>
+        <v>Breakfast stop, 6:30–7:30 AM — at your own expense</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>arang-kel-neelum-valley</v>
+        <v>naran-kaghan-babusar-top</v>
       </c>
       <c r="B6" t="str">
-        <v>Arang Kel</v>
+        <v>Lulusar Lake</v>
       </c>
       <c r="C6">
-        <v>2743</v>
+        <v>3410</v>
       </c>
       <c r="D6" t="str">
-        <v>Days 1–2 · 16:00</v>
+        <v>Day 2 · 09:00</v>
       </c>
       <c r="E6" t="str">
-        <v>arang-kel.jpg</v>
+        <v/>
       </c>
       <c r="F6" t="str">
-        <v>A green shelf above the valley — wooden huts, pine forest, and no road in.</v>
+        <v>The lake the Kunhar river starts from, still and high.</v>
       </c>
       <c r="G6" t="str">
-        <v>One night in a hut — included | Breakfast in the morning | The meadow before the day trippers arrive</v>
+        <v>A stop at the lake on the way up</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>naran-kaghan-babusar-top</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Babusar Top</v>
+      </c>
+      <c r="C7">
+        <v>4173</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Day 2 · 10:30</v>
+      </c>
+      <c r="E7" t="str">
+        <v/>
+      </c>
+      <c r="F7" t="str">
+        <v>The top of the pass, with live snowfall expected in October.</v>
+      </c>
+      <c r="G7" t="str">
+        <v>An hour at the top, 10:30–11:30 AM | Photos at 4,173 m</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>naran-kaghan-babusar-top</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Kaghan</v>
+      </c>
+      <c r="C8">
+        <v>2012</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Day 2 · 15:00</v>
+      </c>
+      <c r="E8" t="str">
+        <v/>
+      </c>
+      <c r="F8" t="str">
+        <v>Back down the valley for a short stay in Kaghan.</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Short stay, 3:00–3:30 PM</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>naran-kaghan-babusar-top</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Balakot</v>
+      </c>
+      <c r="C9">
+        <v>975</v>
+      </c>
+      <c r="D9" t="str">
+        <v>Day 2 · 17:30</v>
+      </c>
+      <c r="E9" t="str">
+        <v/>
+      </c>
+      <c r="F9" t="str">
+        <v>Dinner on the way home, then Islamabad by around 11 PM.</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Dinner at Balakot — included | Leave for Islamabad at 6:30 PM</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G9"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1540,24 +1626,24 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>arang-kel-neelum-valley</v>
+        <v>naran-kaghan-babusar-top</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="str">
-        <v>Midnight departure from Islamabad. Breakfast at Muzaffarabad as the light comes up, then the Neelum valley road all day — tea at Keran, lunch past Sharda. Kel by mid-afternoon, the chairlift across the river, and the last stretch up on foot. Night in a hut at Arang Kel.</v>
+        <v>Report at 5:30 AM at Quaid-e-Azam University; the van leaves at 6:00 sharp, collecting from Kashmir Chowk, Abpara, G-8, H-9, G-13 and 26 Number. Up the Hazara Motorway with breakfast on the way, into Naran by 1 PM, then jeeps to Saif ul Malook Lake. Back in Naran for rafting and the zipline, hotel check-in at 6, and the evening in Naran Bazaar.</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>arang-kel-neelum-valley</v>
+        <v>naran-kaghan-babusar-top</v>
       </c>
       <c r="B3">
         <v>2</v>
       </c>
       <c r="C3" t="str">
-        <v>Out early for the meadow before the day trippers come up. Down the ridge by late morning, back into the van at Kel, and the long drive home. Islamabad the same night.</v>
+        <v>Wake-up call at 5, breakfast at Batakundi, then Lulusar Lake and up to Babusar Top by 10:30 — an hour at the pass, where snow is expected. Down through Kaghan Valley in the afternoon, dinner at Balakot, and back in Islamabad by around 11 PM.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes related to the site trip details and teams
</commit_message>
<xml_diff>
--- a/data/content.xlsx
+++ b/data/content.xlsx
@@ -530,7 +530,7 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F27"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -972,9 +972,109 @@
         <v>https://commons.wikimedia.org/w/index.php?curid=69010681</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>tours/babusar-top.jpg</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Babusar Top, looking towards Naran</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Samikhan86</v>
+      </c>
+      <c r="D23" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E23" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0</v>
+      </c>
+      <c r="F23" t="str">
+        <v>https://commons.wikimedia.org/wiki/File:View_from_babusar_top_towards_naran.jpg</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>tours/batakundi.jpg</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Batakundi, Naran</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Asham Shahzad</v>
+      </c>
+      <c r="D24" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E24" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0</v>
+      </c>
+      <c r="F24" t="str">
+        <v>https://commons.wikimedia.org/wiki/File:Batakundi,_Naran.jpg</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>tours/lulusar.jpg</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Lulusar Lake</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Shahzaib Damn Cruze</v>
+      </c>
+      <c r="D25" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E25" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0</v>
+      </c>
+      <c r="F25" t="str">
+        <v>https://commons.wikimedia.org/wiki/File:Lulusar_Lake_01.jpg</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>tours/kaghan.jpg</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Besar, Kaghan Valley</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Faisal Rafiq</v>
+      </c>
+      <c r="D26" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E26" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0</v>
+      </c>
+      <c r="F26" t="str">
+        <v>https://commons.wikimedia.org/wiki/File:Besar_-_Kaghan_Valley.jpg</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>tours/balakot.jpg</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Balakot, Kaghan Valley</v>
+      </c>
+      <c r="C27" t="str">
+        <v>Mimalkera</v>
+      </c>
+      <c r="D27" t="str">
+        <v>CC BY-SA 4.0</v>
+      </c>
+      <c r="E27" t="str">
+        <v>https://creativecommons.org/licenses/by-sa/4.0</v>
+      </c>
+      <c r="F27" t="str">
+        <v>https://commons.wikimedia.org/wiki/File:Balakot_,_Kaghan_Valley_,_KPK_Pakistan.jpg</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F27"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1501,7 +1601,7 @@
         <v>Day 2 · 06:30</v>
       </c>
       <c r="E5" t="str">
-        <v/>
+        <v>batakundi.jpg</v>
       </c>
       <c r="F5" t="str">
         <v>Wake-up call at five, on the road by half past, breakfast up the valley.</v>
@@ -1524,7 +1624,7 @@
         <v>Day 2 · 09:00</v>
       </c>
       <c r="E6" t="str">
-        <v/>
+        <v>lulusar.jpg</v>
       </c>
       <c r="F6" t="str">
         <v>The lake the Kunhar river starts from, still and high.</v>
@@ -1547,7 +1647,7 @@
         <v>Day 2 · 10:30</v>
       </c>
       <c r="E7" t="str">
-        <v/>
+        <v>babusar-top.jpg</v>
       </c>
       <c r="F7" t="str">
         <v>The top of the pass, with live snowfall expected in October.</v>
@@ -1570,7 +1670,7 @@
         <v>Day 2 · 15:00</v>
       </c>
       <c r="E8" t="str">
-        <v/>
+        <v>kaghan.jpg</v>
       </c>
       <c r="F8" t="str">
         <v>Back down the valley for a short stay in Kaghan.</v>
@@ -1593,7 +1693,7 @@
         <v>Day 2 · 17:30</v>
       </c>
       <c r="E9" t="str">
-        <v/>
+        <v>balakot.jpg</v>
       </c>
       <c r="F9" t="str">
         <v>Dinner on the way home, then Islamabad by around 11 PM.</v>

</xml_diff>